<commit_message>
Estrutura Boletim SDP Analisa 2022
</commit_message>
<xml_diff>
--- a/data-raw/vio_mulher.xlsx
+++ b/data-raw/vio_mulher.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projetos de R\Boletim_sdpa\data-raw\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rafael.rocha\Documents\Projetos R\Boletim_sdpa\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2076" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2093" uniqueCount="26">
   <si>
     <t>Sem</t>
   </si>
@@ -105,7 +105,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -166,9 +166,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Escritório">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -206,7 +206,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Escritório">
       <a:majorFont>
         <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -278,7 +278,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Escritório">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -452,7 +452,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I2068"/>
+  <dimension ref="A1:I2085"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="5" max="5" width="67.5703125" customWidth="1"/>
@@ -60428,6 +60428,499 @@
       </c>
       <c r="I2068">
         <v>178</v>
+      </c>
+    </row>
+    <row r="2069" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2069">
+        <v>2</v>
+      </c>
+      <c r="B2069">
+        <v>4</v>
+      </c>
+      <c r="C2069">
+        <v>12</v>
+      </c>
+      <c r="D2069">
+        <v>2022</v>
+      </c>
+      <c r="E2069" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2069">
+        <v>7</v>
+      </c>
+      <c r="G2069">
+        <v>0</v>
+      </c>
+      <c r="H2069">
+        <v>6</v>
+      </c>
+      <c r="I2069">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2070" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2070">
+        <v>2</v>
+      </c>
+      <c r="B2070">
+        <v>4</v>
+      </c>
+      <c r="C2070">
+        <v>12</v>
+      </c>
+      <c r="D2070">
+        <v>2022</v>
+      </c>
+      <c r="E2070" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2070">
+        <v>6</v>
+      </c>
+      <c r="G2070">
+        <v>5</v>
+      </c>
+      <c r="H2070">
+        <v>9</v>
+      </c>
+      <c r="I2070">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2071" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2071">
+        <v>2</v>
+      </c>
+      <c r="B2071">
+        <v>4</v>
+      </c>
+      <c r="C2071">
+        <v>12</v>
+      </c>
+      <c r="D2071">
+        <v>2022</v>
+      </c>
+      <c r="E2071" t="s">
+        <v>24</v>
+      </c>
+      <c r="F2071">
+        <v>13</v>
+      </c>
+      <c r="G2071">
+        <v>5</v>
+      </c>
+      <c r="H2071">
+        <v>15</v>
+      </c>
+      <c r="I2071">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2072" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2072">
+        <v>2</v>
+      </c>
+      <c r="B2072">
+        <v>4</v>
+      </c>
+      <c r="C2072">
+        <v>12</v>
+      </c>
+      <c r="D2072">
+        <v>2022</v>
+      </c>
+      <c r="E2072" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2072">
+        <v>1</v>
+      </c>
+      <c r="G2072">
+        <v>3</v>
+      </c>
+      <c r="H2072">
+        <v>2</v>
+      </c>
+      <c r="I2072">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2073" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2073">
+        <v>2</v>
+      </c>
+      <c r="B2073">
+        <v>4</v>
+      </c>
+      <c r="C2073">
+        <v>12</v>
+      </c>
+      <c r="D2073">
+        <v>2022</v>
+      </c>
+      <c r="E2073" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2073">
+        <v>7</v>
+      </c>
+      <c r="G2073">
+        <v>11</v>
+      </c>
+      <c r="H2073">
+        <v>23</v>
+      </c>
+      <c r="I2073">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="2074" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2074">
+        <v>2</v>
+      </c>
+      <c r="B2074">
+        <v>4</v>
+      </c>
+      <c r="C2074">
+        <v>12</v>
+      </c>
+      <c r="D2074">
+        <v>2022</v>
+      </c>
+      <c r="E2074" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2074">
+        <v>1660</v>
+      </c>
+      <c r="G2074">
+        <v>741</v>
+      </c>
+      <c r="H2074">
+        <v>2325</v>
+      </c>
+      <c r="I2074">
+        <v>4726</v>
+      </c>
+    </row>
+    <row r="2075" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2075">
+        <v>2</v>
+      </c>
+      <c r="B2075">
+        <v>4</v>
+      </c>
+      <c r="C2075">
+        <v>12</v>
+      </c>
+      <c r="D2075">
+        <v>2022</v>
+      </c>
+      <c r="E2075" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2075">
+        <v>11</v>
+      </c>
+      <c r="G2075">
+        <v>8</v>
+      </c>
+      <c r="H2075">
+        <v>23</v>
+      </c>
+      <c r="I2075">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="2076" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2076">
+        <v>2</v>
+      </c>
+      <c r="B2076">
+        <v>4</v>
+      </c>
+      <c r="C2076">
+        <v>12</v>
+      </c>
+      <c r="D2076">
+        <v>2022</v>
+      </c>
+      <c r="E2076" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2076">
+        <v>2458</v>
+      </c>
+      <c r="G2076">
+        <v>560</v>
+      </c>
+      <c r="H2076">
+        <v>1999</v>
+      </c>
+      <c r="I2076">
+        <v>5017</v>
+      </c>
+    </row>
+    <row r="2077" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2077">
+        <v>2</v>
+      </c>
+      <c r="B2077">
+        <v>4</v>
+      </c>
+      <c r="C2077">
+        <v>12</v>
+      </c>
+      <c r="D2077">
+        <v>2022</v>
+      </c>
+      <c r="E2077" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2077">
+        <v>24</v>
+      </c>
+      <c r="G2077">
+        <v>12</v>
+      </c>
+      <c r="H2077">
+        <v>74</v>
+      </c>
+      <c r="I2077">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="2078" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2078">
+        <v>2</v>
+      </c>
+      <c r="B2078">
+        <v>4</v>
+      </c>
+      <c r="C2078">
+        <v>12</v>
+      </c>
+      <c r="D2078">
+        <v>2022</v>
+      </c>
+      <c r="E2078" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2078">
+        <v>2933</v>
+      </c>
+      <c r="G2078">
+        <v>910</v>
+      </c>
+      <c r="H2078">
+        <v>3789</v>
+      </c>
+      <c r="I2078">
+        <v>7632</v>
+      </c>
+    </row>
+    <row r="2079" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2079">
+        <v>2</v>
+      </c>
+      <c r="B2079">
+        <v>4</v>
+      </c>
+      <c r="C2079">
+        <v>12</v>
+      </c>
+      <c r="D2079">
+        <v>2022</v>
+      </c>
+      <c r="E2079" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2079">
+        <v>61</v>
+      </c>
+      <c r="G2079">
+        <v>25</v>
+      </c>
+      <c r="H2079">
+        <v>105</v>
+      </c>
+      <c r="I2079">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="2080" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2080">
+        <v>2</v>
+      </c>
+      <c r="B2080">
+        <v>4</v>
+      </c>
+      <c r="C2080">
+        <v>12</v>
+      </c>
+      <c r="D2080">
+        <v>2022</v>
+      </c>
+      <c r="E2080" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2080">
+        <v>229</v>
+      </c>
+      <c r="G2080">
+        <v>92</v>
+      </c>
+      <c r="H2080">
+        <v>472</v>
+      </c>
+      <c r="I2080">
+        <v>793</v>
+      </c>
+    </row>
+    <row r="2081" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2081">
+        <v>2</v>
+      </c>
+      <c r="B2081">
+        <v>4</v>
+      </c>
+      <c r="C2081">
+        <v>12</v>
+      </c>
+      <c r="D2081">
+        <v>2022</v>
+      </c>
+      <c r="E2081" t="s">
+        <v>19</v>
+      </c>
+      <c r="F2081">
+        <v>40</v>
+      </c>
+      <c r="G2081">
+        <v>40</v>
+      </c>
+      <c r="H2081">
+        <v>144</v>
+      </c>
+      <c r="I2081">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="2082" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2082">
+        <v>2</v>
+      </c>
+      <c r="B2082">
+        <v>4</v>
+      </c>
+      <c r="C2082">
+        <v>12</v>
+      </c>
+      <c r="D2082">
+        <v>2022</v>
+      </c>
+      <c r="E2082" t="s">
+        <v>20</v>
+      </c>
+      <c r="F2082">
+        <v>10</v>
+      </c>
+      <c r="G2082">
+        <v>7</v>
+      </c>
+      <c r="H2082">
+        <v>24</v>
+      </c>
+      <c r="I2082">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="2083" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2083">
+        <v>2</v>
+      </c>
+      <c r="B2083">
+        <v>4</v>
+      </c>
+      <c r="C2083">
+        <v>12</v>
+      </c>
+      <c r="D2083">
+        <v>2022</v>
+      </c>
+      <c r="E2083" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2083">
+        <v>141</v>
+      </c>
+      <c r="G2083">
+        <v>157</v>
+      </c>
+      <c r="H2083">
+        <v>415</v>
+      </c>
+      <c r="I2083">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="2084" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2084">
+        <v>2</v>
+      </c>
+      <c r="B2084">
+        <v>4</v>
+      </c>
+      <c r="C2084">
+        <v>12</v>
+      </c>
+      <c r="D2084">
+        <v>2022</v>
+      </c>
+      <c r="E2084" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2084">
+        <v>2</v>
+      </c>
+      <c r="G2084">
+        <v>5</v>
+      </c>
+      <c r="H2084">
+        <v>17</v>
+      </c>
+      <c r="I2084">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2085" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2085">
+        <v>2</v>
+      </c>
+      <c r="B2085">
+        <v>4</v>
+      </c>
+      <c r="C2085">
+        <v>12</v>
+      </c>
+      <c r="D2085">
+        <v>2022</v>
+      </c>
+      <c r="E2085" t="s">
+        <v>22</v>
+      </c>
+      <c r="F2085">
+        <v>73</v>
+      </c>
+      <c r="G2085">
+        <v>38</v>
+      </c>
+      <c r="H2085">
+        <v>97</v>
+      </c>
+      <c r="I2085">
+        <v>208</v>
       </c>
     </row>
   </sheetData>

</xml_diff>